<commit_message>
Sync planning SharePoint : S27
</commit_message>
<xml_diff>
--- a/Plannings 2026 S27.xlsx
+++ b/Plannings 2026 S27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9BD0506-81E3-457E-ABEF-F9CA295F4E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{C9BD0506-81E3-457E-ABEF-F9CA295F4E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43903BD4-F6FF-48EB-A0B3-1489F1118A0B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="121">
   <si>
     <t>Planning des salariés du 29/06/2026 au 05/07/2026</t>
   </si>
@@ -379,6 +379,12 @@
   </si>
   <si>
     <t>C. PADEL // LEAGUES</t>
+  </si>
+  <si>
+    <t>18:00/00:30+</t>
+  </si>
+  <si>
+    <t>18:30/01:00+</t>
   </si>
 </sst>
 </file>
@@ -767,7 +773,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -936,6 +942,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4411,8 +4423,8 @@
       <c r="B27" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>55</v>
+      <c r="C27" s="57" t="s">
+        <v>119</v>
       </c>
       <c r="D27" s="50" t="s">
         <v>56</v>
@@ -4581,8 +4593,8 @@
     <row r="39" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="23"/>
       <c r="B39" s="24"/>
-      <c r="C39" s="24" t="s">
-        <v>70</v>
+      <c r="C39" s="58" t="s">
+        <v>120</v>
       </c>
       <c r="D39" s="24"/>
       <c r="E39" s="24" t="s">
@@ -5749,13 +5761,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A6ACA25-883F-46DD-8FAC-0088F0126280}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BC7D462-6616-4EBC-99F4-A6C0B3B6308F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69510268-CC1B-4632-A4CB-6AE030FC320A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29687674-ECD2-46B3-93B0-F504DA9E2663}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DCDBF4C9-CA0B-43D3-A1A0-B0B5BDEF8381}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A18A57DC-3390-445A-B912-A214DBB6007F}"/>
 </file>
</xml_diff>